<commit_message>
einbetten von firmen und bkp
</commit_message>
<xml_diff>
--- a/examples/demo/KONTEN_Übersicht_Moser_Vision (1).xlsx
+++ b/examples/demo/KONTEN_Übersicht_Moser_Vision (1).xlsx
@@ -1050,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BH108"/>
+  <dimension ref="A1:BH369"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="18.42578125" defaultRowHeight="11.25"/>
   <cols>
     <col width="3.28515625" bestFit="1" customWidth="1" style="1" min="1" max="2"/>
@@ -4306,7 +4306,2014 @@
           <t>manually_assigned</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>108</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>109</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>110</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>111</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>112</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>113</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>114</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>115</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>116</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n">
+        <v>117</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>118</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>erfasst</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="n">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="n">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="n">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="n">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="n">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="n">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="n">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="n">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="n">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="n">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="n">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="n">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="n">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="n">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="n">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="n">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="n">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="n">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="n">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="n">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="n">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="n">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="n">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="n">
+        <v>207</v>
+      </c>
+      <c r="B208" t="inlineStr"/>
+      <c r="C208" t="inlineStr"/>
+      <c r="D208" t="inlineStr"/>
+      <c r="E208" t="inlineStr"/>
+    </row>
+    <row r="209">
+      <c r="A209" t="n">
+        <v>208</v>
+      </c>
+      <c r="B209" t="inlineStr"/>
+      <c r="C209" t="inlineStr"/>
+      <c r="D209" t="inlineStr"/>
+      <c r="E209" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" t="n">
+        <v>209</v>
+      </c>
+      <c r="B210" t="inlineStr"/>
+      <c r="C210" t="inlineStr"/>
+      <c r="D210" t="inlineStr"/>
+      <c r="E210" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" t="n">
+        <v>210</v>
+      </c>
+      <c r="B211" t="inlineStr"/>
+      <c r="C211" t="inlineStr"/>
+      <c r="D211" t="inlineStr"/>
+      <c r="E211" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" t="n">
+        <v>211</v>
+      </c>
+      <c r="B212" t="inlineStr"/>
+      <c r="C212" t="inlineStr"/>
+      <c r="D212" t="inlineStr"/>
+      <c r="E212" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" t="n">
+        <v>212</v>
+      </c>
+      <c r="B213" t="inlineStr"/>
+      <c r="C213" t="inlineStr"/>
+      <c r="D213" t="inlineStr"/>
+      <c r="E213" t="inlineStr"/>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>213</v>
+      </c>
+      <c r="B214" t="inlineStr"/>
+      <c r="C214" t="inlineStr"/>
+      <c r="D214" t="inlineStr"/>
+      <c r="E214" t="inlineStr"/>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>214</v>
+      </c>
+      <c r="B215" t="inlineStr"/>
+      <c r="C215" t="inlineStr"/>
+      <c r="D215" t="inlineStr"/>
+      <c r="E215" t="inlineStr"/>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>215</v>
+      </c>
+      <c r="B216" t="inlineStr"/>
+      <c r="C216" t="inlineStr"/>
+      <c r="D216" t="inlineStr"/>
+      <c r="E216" t="inlineStr"/>
+    </row>
+    <row r="217">
+      <c r="A217" t="n">
+        <v>216</v>
+      </c>
+      <c r="B217" t="inlineStr"/>
+      <c r="C217" t="inlineStr"/>
+      <c r="D217" t="inlineStr"/>
+      <c r="E217" t="inlineStr"/>
+    </row>
+    <row r="218">
+      <c r="A218" t="n">
+        <v>217</v>
+      </c>
+      <c r="B218" t="inlineStr"/>
+      <c r="C218" t="inlineStr"/>
+      <c r="D218" t="inlineStr"/>
+      <c r="E218" t="inlineStr"/>
+    </row>
+    <row r="219">
+      <c r="A219" t="n">
+        <v>218</v>
+      </c>
+      <c r="B219" t="inlineStr"/>
+      <c r="C219" t="inlineStr"/>
+      <c r="D219" t="inlineStr"/>
+      <c r="E219" t="inlineStr"/>
+    </row>
+    <row r="220">
+      <c r="A220" t="n">
+        <v>219</v>
+      </c>
+      <c r="B220" t="inlineStr"/>
+      <c r="C220" t="inlineStr"/>
+      <c r="D220" t="inlineStr"/>
+      <c r="E220" t="inlineStr"/>
+    </row>
+    <row r="221">
+      <c r="A221" t="n">
+        <v>220</v>
+      </c>
+      <c r="B221" t="inlineStr"/>
+      <c r="C221" t="inlineStr"/>
+      <c r="D221" t="inlineStr"/>
+      <c r="E221" t="inlineStr"/>
+    </row>
+    <row r="222">
+      <c r="A222" t="n">
+        <v>221</v>
+      </c>
+      <c r="B222" t="inlineStr"/>
+      <c r="C222" t="inlineStr"/>
+      <c r="D222" t="inlineStr"/>
+      <c r="E222" t="inlineStr"/>
+    </row>
+    <row r="223">
+      <c r="A223" t="n">
+        <v>222</v>
+      </c>
+      <c r="B223" t="inlineStr"/>
+      <c r="C223" t="inlineStr"/>
+      <c r="D223" t="inlineStr"/>
+      <c r="E223" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" t="n">
+        <v>223</v>
+      </c>
+      <c r="B224" t="inlineStr"/>
+      <c r="C224" t="inlineStr"/>
+      <c r="D224" t="inlineStr"/>
+      <c r="E224" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" t="n">
+        <v>224</v>
+      </c>
+      <c r="B225" t="inlineStr"/>
+      <c r="C225" t="inlineStr"/>
+      <c r="D225" t="inlineStr"/>
+      <c r="E225" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" t="n">
+        <v>225</v>
+      </c>
+      <c r="B226" t="inlineStr"/>
+      <c r="C226" t="inlineStr"/>
+      <c r="D226" t="inlineStr"/>
+      <c r="E226" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" t="n">
+        <v>226</v>
+      </c>
+      <c r="B227" t="inlineStr"/>
+      <c r="C227" t="inlineStr"/>
+      <c r="D227" t="inlineStr"/>
+      <c r="E227" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" t="n">
+        <v>227</v>
+      </c>
+      <c r="B228" t="inlineStr"/>
+      <c r="C228" t="inlineStr"/>
+      <c r="D228" t="inlineStr"/>
+      <c r="E228" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" t="n">
+        <v>228</v>
+      </c>
+      <c r="B229" t="inlineStr"/>
+      <c r="C229" t="inlineStr"/>
+      <c r="D229" t="inlineStr"/>
+      <c r="E229" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" t="n">
+        <v>229</v>
+      </c>
+      <c r="B230" t="inlineStr"/>
+      <c r="C230" t="inlineStr"/>
+      <c r="D230" t="inlineStr"/>
+      <c r="E230" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" t="n">
+        <v>230</v>
+      </c>
+      <c r="B231" t="inlineStr"/>
+      <c r="C231" t="inlineStr"/>
+      <c r="D231" t="inlineStr"/>
+      <c r="E231" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>231</v>
+      </c>
+      <c r="B232" t="inlineStr"/>
+      <c r="C232" t="inlineStr"/>
+      <c r="D232" t="inlineStr"/>
+      <c r="E232" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>232</v>
+      </c>
+      <c r="B233" t="inlineStr"/>
+      <c r="C233" t="inlineStr"/>
+      <c r="D233" t="inlineStr"/>
+      <c r="E233" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>233</v>
+      </c>
+      <c r="B234" t="inlineStr"/>
+      <c r="C234" t="inlineStr"/>
+      <c r="D234" t="inlineStr"/>
+      <c r="E234" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" t="n">
+        <v>234</v>
+      </c>
+      <c r="B235" t="inlineStr"/>
+      <c r="C235" t="inlineStr"/>
+      <c r="D235" t="inlineStr"/>
+      <c r="E235" t="inlineStr"/>
+    </row>
+    <row r="236">
+      <c r="A236" t="n">
+        <v>235</v>
+      </c>
+      <c r="B236" t="inlineStr"/>
+      <c r="C236" t="inlineStr"/>
+      <c r="D236" t="inlineStr"/>
+      <c r="E236" t="inlineStr"/>
+    </row>
+    <row r="237">
+      <c r="A237" t="n">
+        <v>236</v>
+      </c>
+      <c r="B237" t="inlineStr"/>
+      <c r="C237" t="inlineStr"/>
+      <c r="D237" t="inlineStr"/>
+      <c r="E237" t="inlineStr"/>
+    </row>
+    <row r="238">
+      <c r="A238" t="n">
+        <v>237</v>
+      </c>
+      <c r="B238" t="inlineStr"/>
+      <c r="C238" t="inlineStr"/>
+      <c r="D238" t="inlineStr"/>
+      <c r="E238" t="inlineStr"/>
+    </row>
+    <row r="239">
+      <c r="A239" t="n">
+        <v>238</v>
+      </c>
+      <c r="B239" t="inlineStr"/>
+      <c r="C239" t="inlineStr"/>
+      <c r="D239" t="inlineStr"/>
+      <c r="E239" t="inlineStr"/>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>239</v>
+      </c>
+      <c r="B240" t="inlineStr"/>
+      <c r="C240" t="inlineStr"/>
+      <c r="D240" t="inlineStr"/>
+      <c r="E240" t="inlineStr"/>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>240</v>
+      </c>
+      <c r="B241" t="inlineStr"/>
+      <c r="C241" t="inlineStr"/>
+      <c r="D241" t="inlineStr"/>
+      <c r="E241" t="inlineStr"/>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>241</v>
+      </c>
+      <c r="B242" t="inlineStr"/>
+      <c r="C242" t="inlineStr"/>
+      <c r="D242" t="inlineStr"/>
+      <c r="E242" t="inlineStr"/>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>242</v>
+      </c>
+      <c r="B243" t="inlineStr"/>
+      <c r="C243" t="inlineStr"/>
+      <c r="D243" t="inlineStr"/>
+      <c r="E243" t="inlineStr"/>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>243</v>
+      </c>
+      <c r="B244" t="inlineStr"/>
+      <c r="C244" t="inlineStr"/>
+      <c r="D244" t="inlineStr"/>
+      <c r="E244" t="inlineStr"/>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>244</v>
+      </c>
+      <c r="B245" t="inlineStr"/>
+      <c r="C245" t="inlineStr"/>
+      <c r="D245" t="inlineStr"/>
+      <c r="E245" t="inlineStr"/>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>245</v>
+      </c>
+      <c r="B246" t="inlineStr"/>
+      <c r="C246" t="inlineStr"/>
+      <c r="D246" t="inlineStr"/>
+      <c r="E246" t="inlineStr"/>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>246</v>
+      </c>
+      <c r="B247" t="inlineStr"/>
+      <c r="C247" t="inlineStr"/>
+      <c r="D247" t="inlineStr"/>
+      <c r="E247" t="inlineStr"/>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>247</v>
+      </c>
+      <c r="B248" t="inlineStr"/>
+      <c r="C248" t="inlineStr"/>
+      <c r="D248" t="inlineStr"/>
+      <c r="E248" t="inlineStr"/>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>248</v>
+      </c>
+      <c r="B249" t="inlineStr"/>
+      <c r="C249" t="inlineStr"/>
+      <c r="D249" t="inlineStr"/>
+      <c r="E249" t="inlineStr"/>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>249</v>
+      </c>
+      <c r="B250" t="inlineStr"/>
+      <c r="C250" t="inlineStr"/>
+      <c r="D250" t="inlineStr"/>
+      <c r="E250" t="inlineStr"/>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>250</v>
+      </c>
+      <c r="B251" t="inlineStr"/>
+      <c r="C251" t="inlineStr"/>
+      <c r="D251" t="inlineStr"/>
+      <c r="E251" t="inlineStr"/>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>251</v>
+      </c>
+      <c r="B252" t="inlineStr"/>
+      <c r="C252" t="inlineStr"/>
+      <c r="D252" t="inlineStr"/>
+      <c r="E252" t="inlineStr"/>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>252</v>
+      </c>
+      <c r="B253" t="inlineStr"/>
+      <c r="C253" t="inlineStr"/>
+      <c r="D253" t="inlineStr"/>
+      <c r="E253" t="inlineStr"/>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>253</v>
+      </c>
+      <c r="B254" t="inlineStr"/>
+      <c r="C254" t="inlineStr"/>
+      <c r="D254" t="inlineStr"/>
+      <c r="E254" t="inlineStr"/>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
+        <v>254</v>
+      </c>
+      <c r="B255" t="inlineStr"/>
+      <c r="C255" t="inlineStr"/>
+      <c r="D255" t="inlineStr"/>
+      <c r="E255" t="inlineStr"/>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>255</v>
+      </c>
+      <c r="B256" t="inlineStr"/>
+      <c r="C256" t="inlineStr"/>
+      <c r="D256" t="inlineStr"/>
+      <c r="E256" t="inlineStr"/>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>256</v>
+      </c>
+      <c r="B257" t="inlineStr"/>
+      <c r="C257" t="inlineStr"/>
+      <c r="D257" t="inlineStr"/>
+      <c r="E257" t="inlineStr"/>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>257</v>
+      </c>
+      <c r="B258" t="inlineStr"/>
+      <c r="C258" t="inlineStr"/>
+      <c r="D258" t="inlineStr"/>
+      <c r="E258" t="inlineStr"/>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>258</v>
+      </c>
+      <c r="B259" t="inlineStr"/>
+      <c r="C259" t="inlineStr"/>
+      <c r="D259" t="inlineStr"/>
+      <c r="E259" t="inlineStr"/>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>259</v>
+      </c>
+      <c r="B260" t="inlineStr"/>
+      <c r="C260" t="inlineStr"/>
+      <c r="D260" t="inlineStr"/>
+      <c r="E260" t="inlineStr"/>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>260</v>
+      </c>
+      <c r="B261" t="inlineStr"/>
+      <c r="C261" t="inlineStr"/>
+      <c r="D261" t="inlineStr"/>
+      <c r="E261" t="inlineStr"/>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>261</v>
+      </c>
+      <c r="B262" t="inlineStr"/>
+      <c r="C262" t="inlineStr"/>
+      <c r="D262" t="inlineStr"/>
+      <c r="E262" t="inlineStr"/>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>262</v>
+      </c>
+      <c r="B263" t="inlineStr"/>
+      <c r="C263" t="inlineStr"/>
+      <c r="D263" t="inlineStr"/>
+      <c r="E263" t="inlineStr"/>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>263</v>
+      </c>
+      <c r="B264" t="inlineStr"/>
+      <c r="C264" t="inlineStr"/>
+      <c r="D264" t="inlineStr"/>
+      <c r="E264" t="inlineStr"/>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>264</v>
+      </c>
+      <c r="B265" t="inlineStr"/>
+      <c r="C265" t="inlineStr"/>
+      <c r="D265" t="inlineStr"/>
+      <c r="E265" t="inlineStr"/>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>265</v>
+      </c>
+      <c r="B266" t="inlineStr"/>
+      <c r="C266" t="inlineStr"/>
+      <c r="D266" t="inlineStr"/>
+      <c r="E266" t="inlineStr"/>
+    </row>
+    <row r="267">
+      <c r="A267" t="n">
+        <v>266</v>
+      </c>
+      <c r="B267" t="inlineStr"/>
+      <c r="C267" t="inlineStr"/>
+      <c r="D267" t="inlineStr"/>
+      <c r="E267" t="inlineStr"/>
+    </row>
+    <row r="268">
+      <c r="A268" t="n">
+        <v>267</v>
+      </c>
+      <c r="B268" t="inlineStr"/>
+      <c r="C268" t="inlineStr"/>
+      <c r="D268" t="inlineStr"/>
+      <c r="E268" t="inlineStr"/>
+    </row>
+    <row r="269">
+      <c r="A269" t="n">
+        <v>268</v>
+      </c>
+      <c r="B269" t="inlineStr"/>
+      <c r="C269" t="inlineStr"/>
+      <c r="D269" t="inlineStr"/>
+      <c r="E269" t="inlineStr"/>
+    </row>
+    <row r="270">
+      <c r="A270" t="n">
+        <v>269</v>
+      </c>
+      <c r="B270" t="inlineStr"/>
+      <c r="C270" t="inlineStr"/>
+      <c r="D270" t="inlineStr"/>
+      <c r="E270" t="inlineStr"/>
+    </row>
+    <row r="271">
+      <c r="A271" t="n">
+        <v>270</v>
+      </c>
+      <c r="B271" t="inlineStr"/>
+      <c r="C271" t="inlineStr"/>
+      <c r="D271" t="inlineStr"/>
+      <c r="E271" t="inlineStr"/>
+    </row>
+    <row r="272">
+      <c r="A272" t="n">
+        <v>271</v>
+      </c>
+      <c r="B272" t="inlineStr"/>
+      <c r="C272" t="inlineStr"/>
+      <c r="D272" t="inlineStr"/>
+      <c r="E272" t="inlineStr"/>
+    </row>
+    <row r="273">
+      <c r="A273" t="n">
+        <v>272</v>
+      </c>
+      <c r="B273" t="inlineStr"/>
+      <c r="C273" t="inlineStr"/>
+      <c r="D273" t="inlineStr"/>
+      <c r="E273" t="inlineStr"/>
+    </row>
+    <row r="274">
+      <c r="A274" t="n">
+        <v>273</v>
+      </c>
+      <c r="B274" t="inlineStr"/>
+      <c r="C274" t="inlineStr"/>
+      <c r="D274" t="inlineStr"/>
+      <c r="E274" t="inlineStr"/>
+    </row>
+    <row r="275">
+      <c r="A275" t="n">
+        <v>274</v>
+      </c>
+      <c r="B275" t="inlineStr"/>
+      <c r="C275" t="inlineStr"/>
+      <c r="D275" t="inlineStr"/>
+      <c r="E275" t="inlineStr"/>
+    </row>
+    <row r="276">
+      <c r="A276" t="n">
+        <v>275</v>
+      </c>
+      <c r="B276" t="inlineStr"/>
+      <c r="C276" t="inlineStr"/>
+      <c r="D276" t="inlineStr"/>
+      <c r="E276" t="inlineStr"/>
+    </row>
+    <row r="277">
+      <c r="A277" t="n">
+        <v>276</v>
+      </c>
+      <c r="B277" t="inlineStr"/>
+      <c r="C277" t="inlineStr"/>
+      <c r="D277" t="inlineStr"/>
+      <c r="E277" t="inlineStr"/>
+    </row>
+    <row r="278">
+      <c r="A278" t="n">
+        <v>277</v>
+      </c>
+      <c r="B278" t="inlineStr"/>
+      <c r="C278" t="inlineStr"/>
+      <c r="D278" t="inlineStr"/>
+      <c r="E278" t="inlineStr"/>
+    </row>
+    <row r="279">
+      <c r="A279" t="n">
+        <v>278</v>
+      </c>
+      <c r="B279" t="inlineStr"/>
+      <c r="C279" t="inlineStr"/>
+      <c r="D279" t="inlineStr"/>
+      <c r="E279" t="inlineStr"/>
+    </row>
+    <row r="280">
+      <c r="A280" t="n">
+        <v>279</v>
+      </c>
+      <c r="B280" t="inlineStr"/>
+      <c r="C280" t="inlineStr"/>
+      <c r="D280" t="inlineStr"/>
+      <c r="E280" t="inlineStr"/>
+    </row>
+    <row r="281">
+      <c r="A281" t="n">
+        <v>280</v>
+      </c>
+      <c r="B281" t="inlineStr"/>
+      <c r="C281" t="inlineStr"/>
+      <c r="D281" t="inlineStr"/>
+      <c r="E281" t="inlineStr"/>
+    </row>
+    <row r="282">
+      <c r="A282" t="n">
+        <v>281</v>
+      </c>
+      <c r="B282" t="inlineStr"/>
+      <c r="C282" t="inlineStr"/>
+      <c r="D282" t="inlineStr"/>
+      <c r="E282" t="inlineStr"/>
+    </row>
+    <row r="283">
+      <c r="A283" t="n">
+        <v>282</v>
+      </c>
+      <c r="B283" t="inlineStr"/>
+      <c r="C283" t="inlineStr"/>
+      <c r="D283" t="inlineStr"/>
+      <c r="E283" t="inlineStr"/>
+    </row>
+    <row r="284">
+      <c r="A284" t="n">
+        <v>283</v>
+      </c>
+      <c r="B284" t="inlineStr"/>
+      <c r="C284" t="inlineStr"/>
+      <c r="D284" t="inlineStr"/>
+      <c r="E284" t="inlineStr"/>
+    </row>
+    <row r="285">
+      <c r="A285" t="n">
+        <v>284</v>
+      </c>
+      <c r="B285" t="inlineStr"/>
+      <c r="C285" t="inlineStr"/>
+      <c r="D285" t="inlineStr"/>
+      <c r="E285" t="inlineStr"/>
+    </row>
+    <row r="286">
+      <c r="A286" t="n">
+        <v>285</v>
+      </c>
+      <c r="B286" t="inlineStr"/>
+      <c r="C286" t="inlineStr"/>
+      <c r="D286" t="inlineStr"/>
+      <c r="E286" t="inlineStr"/>
+    </row>
+    <row r="287">
+      <c r="A287" t="n">
+        <v>286</v>
+      </c>
+      <c r="B287" t="inlineStr"/>
+      <c r="C287" t="inlineStr"/>
+      <c r="D287" t="inlineStr"/>
+      <c r="E287" t="inlineStr"/>
+    </row>
+    <row r="288">
+      <c r="A288" t="n">
+        <v>287</v>
+      </c>
+      <c r="B288" t="inlineStr"/>
+      <c r="C288" t="inlineStr"/>
+      <c r="D288" t="inlineStr"/>
+      <c r="E288" t="inlineStr"/>
+    </row>
+    <row r="289">
+      <c r="A289" t="n">
+        <v>288</v>
+      </c>
+      <c r="B289" t="inlineStr"/>
+      <c r="C289" t="inlineStr"/>
+      <c r="D289" t="inlineStr"/>
+      <c r="E289" t="inlineStr"/>
+    </row>
+    <row r="290">
+      <c r="A290" t="n">
+        <v>289</v>
+      </c>
+      <c r="B290" t="inlineStr"/>
+      <c r="C290" t="inlineStr"/>
+      <c r="D290" t="inlineStr"/>
+      <c r="E290" t="inlineStr"/>
+    </row>
+    <row r="291">
+      <c r="A291" t="n">
+        <v>290</v>
+      </c>
+      <c r="B291" t="inlineStr"/>
+      <c r="C291" t="inlineStr"/>
+      <c r="D291" t="inlineStr"/>
+      <c r="E291" t="inlineStr"/>
+    </row>
+    <row r="292">
+      <c r="A292" t="n">
+        <v>291</v>
+      </c>
+      <c r="B292" t="inlineStr"/>
+      <c r="C292" t="inlineStr"/>
+      <c r="D292" t="inlineStr"/>
+      <c r="E292" t="inlineStr"/>
+    </row>
+    <row r="293">
+      <c r="A293" t="n">
+        <v>292</v>
+      </c>
+      <c r="B293" t="inlineStr"/>
+      <c r="C293" t="inlineStr"/>
+      <c r="D293" t="inlineStr"/>
+      <c r="E293" t="inlineStr"/>
+    </row>
+    <row r="294">
+      <c r="A294" t="n">
+        <v>293</v>
+      </c>
+      <c r="B294" t="inlineStr"/>
+      <c r="C294" t="inlineStr"/>
+      <c r="D294" t="inlineStr"/>
+      <c r="E294" t="inlineStr"/>
+    </row>
+    <row r="295">
+      <c r="A295" t="n">
+        <v>294</v>
+      </c>
+      <c r="B295" t="inlineStr"/>
+      <c r="C295" t="inlineStr"/>
+      <c r="D295" t="inlineStr"/>
+      <c r="E295" t="inlineStr"/>
+    </row>
+    <row r="296">
+      <c r="A296" t="n">
+        <v>295</v>
+      </c>
+      <c r="B296" t="inlineStr"/>
+      <c r="C296" t="inlineStr"/>
+      <c r="D296" t="inlineStr"/>
+      <c r="E296" t="inlineStr"/>
+    </row>
+    <row r="297">
+      <c r="A297" t="n">
+        <v>296</v>
+      </c>
+      <c r="B297" t="inlineStr"/>
+      <c r="C297" t="inlineStr"/>
+      <c r="D297" t="inlineStr"/>
+      <c r="E297" t="inlineStr"/>
+    </row>
+    <row r="298">
+      <c r="A298" t="n">
+        <v>297</v>
+      </c>
+      <c r="B298" t="inlineStr"/>
+      <c r="C298" t="inlineStr"/>
+      <c r="D298" t="inlineStr"/>
+      <c r="E298" t="inlineStr"/>
+    </row>
+    <row r="299">
+      <c r="A299" t="n">
+        <v>298</v>
+      </c>
+      <c r="B299" t="inlineStr"/>
+      <c r="C299" t="inlineStr"/>
+      <c r="D299" t="inlineStr"/>
+      <c r="E299" t="inlineStr"/>
+    </row>
+    <row r="300">
+      <c r="A300" t="n">
+        <v>299</v>
+      </c>
+      <c r="B300" t="inlineStr"/>
+      <c r="C300" t="inlineStr"/>
+      <c r="D300" t="inlineStr"/>
+      <c r="E300" t="inlineStr"/>
+    </row>
+    <row r="301">
+      <c r="A301" t="n">
+        <v>300</v>
+      </c>
+      <c r="B301" t="inlineStr"/>
+      <c r="C301" t="inlineStr"/>
+      <c r="D301" t="inlineStr"/>
+      <c r="E301" t="inlineStr"/>
+    </row>
+    <row r="302">
+      <c r="A302" t="n">
+        <v>301</v>
+      </c>
+      <c r="B302" t="inlineStr"/>
+      <c r="C302" t="inlineStr"/>
+      <c r="D302" t="inlineStr"/>
+      <c r="E302" t="inlineStr"/>
+    </row>
+    <row r="303">
+      <c r="A303" t="n">
+        <v>302</v>
+      </c>
+      <c r="B303" t="inlineStr"/>
+      <c r="C303" t="inlineStr"/>
+      <c r="D303" t="inlineStr"/>
+      <c r="E303" t="inlineStr"/>
+    </row>
+    <row r="304">
+      <c r="A304" t="n">
+        <v>303</v>
+      </c>
+      <c r="B304" t="inlineStr"/>
+      <c r="C304" t="inlineStr"/>
+      <c r="D304" t="inlineStr"/>
+      <c r="E304" t="inlineStr"/>
+    </row>
+    <row r="305">
+      <c r="A305" t="n">
+        <v>304</v>
+      </c>
+      <c r="B305" t="inlineStr"/>
+      <c r="C305" t="inlineStr"/>
+      <c r="D305" t="inlineStr"/>
+      <c r="E305" t="inlineStr"/>
+    </row>
+    <row r="306">
+      <c r="A306" t="n">
+        <v>305</v>
+      </c>
+      <c r="B306" t="inlineStr"/>
+      <c r="C306" t="inlineStr"/>
+      <c r="D306" t="inlineStr"/>
+      <c r="E306" t="inlineStr"/>
+    </row>
+    <row r="307">
+      <c r="A307" t="n">
+        <v>306</v>
+      </c>
+      <c r="B307" t="inlineStr"/>
+      <c r="C307" t="inlineStr"/>
+      <c r="D307" t="inlineStr"/>
+      <c r="E307" t="inlineStr"/>
+    </row>
+    <row r="308">
+      <c r="A308" t="n">
+        <v>307</v>
+      </c>
+      <c r="B308" t="inlineStr"/>
+      <c r="C308" t="inlineStr"/>
+      <c r="D308" t="inlineStr"/>
+      <c r="E308" t="inlineStr"/>
+    </row>
+    <row r="309">
+      <c r="A309" t="n">
+        <v>308</v>
+      </c>
+      <c r="B309" t="inlineStr"/>
+      <c r="C309" t="inlineStr"/>
+      <c r="D309" t="inlineStr"/>
+      <c r="E309" t="inlineStr"/>
+    </row>
+    <row r="310">
+      <c r="A310" t="n">
+        <v>309</v>
+      </c>
+      <c r="B310" t="inlineStr"/>
+      <c r="C310" t="inlineStr"/>
+      <c r="D310" t="inlineStr"/>
+      <c r="E310" t="inlineStr"/>
+    </row>
+    <row r="311">
+      <c r="A311" t="n">
+        <v>310</v>
+      </c>
+      <c r="B311" t="inlineStr"/>
+      <c r="C311" t="inlineStr"/>
+      <c r="D311" t="inlineStr"/>
+      <c r="E311" t="inlineStr"/>
+    </row>
+    <row r="312">
+      <c r="A312" t="n">
+        <v>311</v>
+      </c>
+      <c r="B312" t="inlineStr"/>
+      <c r="C312" t="inlineStr"/>
+      <c r="D312" t="inlineStr"/>
+      <c r="E312" t="inlineStr"/>
+    </row>
+    <row r="313">
+      <c r="A313" t="n">
+        <v>312</v>
+      </c>
+      <c r="B313" t="inlineStr"/>
+      <c r="C313" t="inlineStr"/>
+      <c r="D313" t="inlineStr"/>
+      <c r="E313" t="inlineStr"/>
+    </row>
+    <row r="314">
+      <c r="A314" t="n">
+        <v>313</v>
+      </c>
+      <c r="B314" t="inlineStr"/>
+      <c r="C314" t="inlineStr"/>
+      <c r="D314" t="inlineStr"/>
+      <c r="E314" t="inlineStr"/>
+    </row>
+    <row r="315">
+      <c r="A315" t="n">
+        <v>314</v>
+      </c>
+      <c r="B315" t="inlineStr"/>
+      <c r="C315" t="inlineStr"/>
+      <c r="D315" t="inlineStr"/>
+      <c r="E315" t="inlineStr"/>
+    </row>
+    <row r="316">
+      <c r="A316" t="n">
+        <v>315</v>
+      </c>
+      <c r="B316" t="inlineStr"/>
+      <c r="C316" t="inlineStr"/>
+      <c r="D316" t="inlineStr"/>
+      <c r="E316" t="inlineStr"/>
+    </row>
+    <row r="317">
+      <c r="A317" t="n">
+        <v>316</v>
+      </c>
+      <c r="B317" t="inlineStr"/>
+      <c r="C317" t="inlineStr"/>
+      <c r="D317" t="inlineStr"/>
+      <c r="E317" t="inlineStr"/>
+    </row>
+    <row r="318">
+      <c r="A318" t="n">
+        <v>317</v>
+      </c>
+      <c r="B318" t="inlineStr"/>
+      <c r="C318" t="inlineStr"/>
+      <c r="D318" t="inlineStr"/>
+      <c r="E318" t="inlineStr"/>
+    </row>
+    <row r="319">
+      <c r="A319" t="n">
+        <v>318</v>
+      </c>
+      <c r="B319" t="inlineStr"/>
+      <c r="C319" t="inlineStr"/>
+      <c r="D319" t="inlineStr"/>
+      <c r="E319" t="inlineStr"/>
+    </row>
+    <row r="320">
+      <c r="A320" t="n">
+        <v>319</v>
+      </c>
+      <c r="B320" t="inlineStr"/>
+      <c r="C320" t="inlineStr"/>
+      <c r="D320" t="inlineStr"/>
+      <c r="E320" t="inlineStr"/>
+    </row>
+    <row r="321">
+      <c r="A321" t="n">
+        <v>320</v>
+      </c>
+      <c r="B321" t="inlineStr"/>
+      <c r="C321" t="inlineStr"/>
+      <c r="D321" t="inlineStr"/>
+      <c r="E321" t="inlineStr"/>
+    </row>
+    <row r="322">
+      <c r="A322" t="n">
+        <v>321</v>
+      </c>
+      <c r="B322" t="inlineStr"/>
+      <c r="C322" t="inlineStr"/>
+      <c r="D322" t="inlineStr"/>
+      <c r="E322" t="inlineStr"/>
+    </row>
+    <row r="323">
+      <c r="A323" t="n">
+        <v>322</v>
+      </c>
+      <c r="B323" t="inlineStr"/>
+      <c r="C323" t="inlineStr"/>
+      <c r="D323" t="inlineStr"/>
+      <c r="E323" t="inlineStr"/>
+    </row>
+    <row r="324">
+      <c r="A324" t="n">
+        <v>323</v>
+      </c>
+      <c r="B324" t="inlineStr"/>
+      <c r="C324" t="inlineStr"/>
+      <c r="D324" t="inlineStr"/>
+      <c r="E324" t="inlineStr"/>
+    </row>
+    <row r="325">
+      <c r="A325" t="n">
+        <v>324</v>
+      </c>
+      <c r="B325" t="inlineStr"/>
+      <c r="C325" t="inlineStr"/>
+      <c r="D325" t="inlineStr"/>
+      <c r="E325" t="inlineStr"/>
+    </row>
+    <row r="326">
+      <c r="A326" t="n">
+        <v>325</v>
+      </c>
+      <c r="B326" t="inlineStr"/>
+      <c r="C326" t="inlineStr"/>
+      <c r="D326" t="inlineStr"/>
+      <c r="E326" t="inlineStr"/>
+    </row>
+    <row r="327">
+      <c r="A327" t="n">
+        <v>326</v>
+      </c>
+      <c r="B327" t="inlineStr"/>
+      <c r="C327" t="inlineStr"/>
+      <c r="D327" t="inlineStr"/>
+      <c r="E327" t="inlineStr"/>
+    </row>
+    <row r="328">
+      <c r="A328" t="n">
+        <v>327</v>
+      </c>
+      <c r="B328" t="inlineStr"/>
+      <c r="C328" t="inlineStr"/>
+      <c r="D328" t="inlineStr"/>
+      <c r="E328" t="inlineStr"/>
+    </row>
+    <row r="329">
+      <c r="A329" t="n">
+        <v>328</v>
+      </c>
+      <c r="B329" t="inlineStr"/>
+      <c r="C329" t="inlineStr"/>
+      <c r="D329" t="inlineStr"/>
+      <c r="E329" t="inlineStr"/>
+    </row>
+    <row r="330">
+      <c r="A330" t="n">
+        <v>329</v>
+      </c>
+      <c r="B330" t="inlineStr"/>
+      <c r="C330" t="inlineStr"/>
+      <c r="D330" t="inlineStr"/>
+      <c r="E330" t="inlineStr"/>
+    </row>
+    <row r="331">
+      <c r="A331" t="n">
+        <v>330</v>
+      </c>
+      <c r="B331" t="inlineStr"/>
+      <c r="C331" t="inlineStr"/>
+      <c r="D331" t="inlineStr"/>
+      <c r="E331" t="inlineStr"/>
+    </row>
+    <row r="332">
+      <c r="A332" t="n">
+        <v>331</v>
+      </c>
+      <c r="B332" t="inlineStr"/>
+      <c r="C332" t="inlineStr"/>
+      <c r="D332" t="inlineStr"/>
+      <c r="E332" t="inlineStr"/>
+    </row>
+    <row r="333">
+      <c r="A333" t="n">
+        <v>332</v>
+      </c>
+      <c r="B333" t="inlineStr"/>
+      <c r="C333" t="inlineStr"/>
+      <c r="D333" t="inlineStr"/>
+      <c r="E333" t="inlineStr"/>
+    </row>
+    <row r="334">
+      <c r="A334" t="n">
+        <v>333</v>
+      </c>
+      <c r="B334" t="inlineStr"/>
+      <c r="C334" t="inlineStr"/>
+      <c r="D334" t="inlineStr"/>
+      <c r="E334" t="inlineStr"/>
+    </row>
+    <row r="335">
+      <c r="A335" t="n">
+        <v>334</v>
+      </c>
+      <c r="B335" t="inlineStr"/>
+      <c r="C335" t="inlineStr"/>
+      <c r="D335" t="inlineStr"/>
+      <c r="E335" t="inlineStr"/>
+    </row>
+    <row r="336">
+      <c r="A336" t="n">
+        <v>335</v>
+      </c>
+      <c r="B336" t="inlineStr"/>
+      <c r="C336" t="inlineStr"/>
+      <c r="D336" t="inlineStr"/>
+      <c r="E336" t="inlineStr"/>
+    </row>
+    <row r="337">
+      <c r="A337" t="n">
+        <v>336</v>
+      </c>
+      <c r="B337" t="inlineStr"/>
+      <c r="C337" t="inlineStr"/>
+      <c r="D337" t="inlineStr"/>
+      <c r="E337" t="inlineStr"/>
+    </row>
+    <row r="338">
+      <c r="A338" t="n">
+        <v>337</v>
+      </c>
+      <c r="B338" t="inlineStr"/>
+      <c r="C338" t="inlineStr"/>
+      <c r="D338" t="inlineStr"/>
+      <c r="E338" t="inlineStr"/>
+    </row>
+    <row r="339">
+      <c r="A339" t="n">
+        <v>338</v>
+      </c>
+      <c r="B339" t="inlineStr"/>
+      <c r="C339" t="inlineStr"/>
+      <c r="D339" t="inlineStr"/>
+      <c r="E339" t="inlineStr"/>
+    </row>
+    <row r="340">
+      <c r="A340" t="n">
+        <v>339</v>
+      </c>
+      <c r="B340" t="inlineStr"/>
+      <c r="C340" t="inlineStr"/>
+      <c r="D340" t="inlineStr"/>
+      <c r="E340" t="inlineStr"/>
+    </row>
+    <row r="341">
+      <c r="A341" t="n">
+        <v>340</v>
+      </c>
+      <c r="B341" t="inlineStr"/>
+      <c r="C341" t="inlineStr"/>
+      <c r="D341" t="inlineStr"/>
+      <c r="E341" t="inlineStr"/>
+    </row>
+    <row r="342">
+      <c r="A342" t="n">
+        <v>341</v>
+      </c>
+      <c r="B342" t="inlineStr"/>
+      <c r="C342" t="inlineStr"/>
+      <c r="D342" t="inlineStr"/>
+      <c r="E342" t="inlineStr"/>
+    </row>
+    <row r="343">
+      <c r="A343" t="n">
+        <v>342</v>
+      </c>
+      <c r="B343" t="inlineStr"/>
+      <c r="C343" t="inlineStr"/>
+      <c r="D343" t="inlineStr"/>
+      <c r="E343" t="inlineStr"/>
+    </row>
+    <row r="344">
+      <c r="A344" t="n">
+        <v>343</v>
+      </c>
+      <c r="B344" t="inlineStr"/>
+      <c r="C344" t="inlineStr"/>
+      <c r="D344" t="inlineStr"/>
+      <c r="E344" t="inlineStr"/>
+    </row>
+    <row r="345">
+      <c r="A345" t="n">
+        <v>344</v>
+      </c>
+      <c r="B345" t="inlineStr"/>
+      <c r="C345" t="inlineStr"/>
+      <c r="D345" t="inlineStr"/>
+      <c r="E345" t="inlineStr"/>
+    </row>
+    <row r="346">
+      <c r="A346" t="n">
+        <v>345</v>
+      </c>
+      <c r="B346" t="inlineStr"/>
+      <c r="C346" t="inlineStr"/>
+      <c r="D346" t="inlineStr"/>
+      <c r="E346" t="inlineStr"/>
+    </row>
+    <row r="347">
+      <c r="A347" t="n">
+        <v>346</v>
+      </c>
+      <c r="B347" t="inlineStr"/>
+      <c r="C347" t="inlineStr"/>
+      <c r="D347" t="inlineStr"/>
+      <c r="E347" t="inlineStr"/>
+    </row>
+    <row r="348">
+      <c r="A348" t="n">
+        <v>347</v>
+      </c>
+      <c r="B348" t="inlineStr"/>
+      <c r="C348" t="inlineStr"/>
+      <c r="D348" t="inlineStr"/>
+      <c r="E348" t="inlineStr"/>
+    </row>
+    <row r="349">
+      <c r="A349" t="n">
+        <v>348</v>
+      </c>
+      <c r="B349" t="inlineStr"/>
+      <c r="C349" t="inlineStr"/>
+      <c r="D349" t="inlineStr"/>
+      <c r="E349" t="inlineStr"/>
+    </row>
+    <row r="350">
+      <c r="A350" t="n">
+        <v>349</v>
+      </c>
+      <c r="B350" t="inlineStr"/>
+      <c r="C350" t="inlineStr"/>
+      <c r="D350" t="inlineStr"/>
+      <c r="E350" t="inlineStr"/>
+    </row>
+    <row r="351">
+      <c r="A351" t="n">
+        <v>350</v>
+      </c>
+      <c r="B351" t="inlineStr"/>
+      <c r="C351" t="inlineStr"/>
+      <c r="D351" t="inlineStr"/>
+      <c r="E351" t="inlineStr"/>
+    </row>
+    <row r="352">
+      <c r="A352" t="n">
+        <v>351</v>
+      </c>
+      <c r="B352" t="inlineStr"/>
+      <c r="C352" t="inlineStr"/>
+      <c r="D352" t="inlineStr"/>
+      <c r="E352" t="inlineStr"/>
+    </row>
+    <row r="353">
+      <c r="A353" t="n">
+        <v>352</v>
+      </c>
+      <c r="B353" t="inlineStr"/>
+      <c r="C353" t="inlineStr"/>
+      <c r="D353" t="inlineStr"/>
+      <c r="E353" t="inlineStr"/>
+    </row>
+    <row r="354">
+      <c r="A354" t="n">
+        <v>353</v>
+      </c>
+      <c r="B354" t="inlineStr"/>
+      <c r="C354" t="inlineStr"/>
+      <c r="D354" t="inlineStr"/>
+      <c r="E354" t="inlineStr"/>
+    </row>
+    <row r="355">
+      <c r="A355" t="n">
+        <v>354</v>
+      </c>
+      <c r="B355" t="inlineStr"/>
+      <c r="C355" t="inlineStr"/>
+      <c r="D355" t="inlineStr"/>
+      <c r="E355" t="inlineStr"/>
+    </row>
+    <row r="356">
+      <c r="A356" t="n">
+        <v>355</v>
+      </c>
+      <c r="B356" t="inlineStr"/>
+      <c r="C356" t="inlineStr"/>
+      <c r="D356" t="inlineStr"/>
+      <c r="E356" t="inlineStr"/>
+    </row>
+    <row r="357">
+      <c r="A357" t="n">
+        <v>356</v>
+      </c>
+      <c r="B357" t="inlineStr"/>
+      <c r="C357" t="inlineStr"/>
+      <c r="D357" t="inlineStr"/>
+      <c r="E357" t="inlineStr"/>
+    </row>
+    <row r="358">
+      <c r="A358" t="n">
+        <v>357</v>
+      </c>
+      <c r="B358" t="inlineStr"/>
+      <c r="C358" t="inlineStr"/>
+      <c r="D358" t="inlineStr"/>
+      <c r="E358" t="inlineStr"/>
+    </row>
+    <row r="359">
+      <c r="A359" t="n">
+        <v>358</v>
+      </c>
+      <c r="B359" t="inlineStr"/>
+      <c r="C359" t="inlineStr"/>
+      <c r="D359" t="inlineStr"/>
+      <c r="E359" t="inlineStr"/>
+    </row>
+    <row r="360">
+      <c r="A360" t="n">
+        <v>359</v>
+      </c>
+      <c r="B360" t="inlineStr"/>
+      <c r="C360" t="inlineStr"/>
+      <c r="D360" t="inlineStr"/>
+      <c r="E360" t="inlineStr"/>
+    </row>
+    <row r="361">
+      <c r="A361" t="n">
+        <v>360</v>
+      </c>
+      <c r="B361" t="inlineStr"/>
+      <c r="C361" t="inlineStr"/>
+      <c r="D361" t="inlineStr"/>
+      <c r="E361" t="inlineStr"/>
+    </row>
+    <row r="362">
+      <c r="A362" t="n">
+        <v>361</v>
+      </c>
+      <c r="B362" t="inlineStr"/>
+      <c r="C362" t="inlineStr"/>
+      <c r="D362" t="inlineStr"/>
+      <c r="E362" t="inlineStr"/>
+    </row>
+    <row r="363">
+      <c r="A363" t="n">
+        <v>362</v>
+      </c>
+      <c r="B363" t="inlineStr"/>
+      <c r="C363" t="inlineStr"/>
+      <c r="D363" t="inlineStr"/>
+      <c r="E363" t="inlineStr"/>
+    </row>
+    <row r="364">
+      <c r="A364" t="n">
+        <v>363</v>
+      </c>
+      <c r="B364" t="inlineStr"/>
+      <c r="C364" t="inlineStr"/>
+      <c r="D364" t="inlineStr"/>
+      <c r="E364" t="inlineStr"/>
+    </row>
+    <row r="365">
+      <c r="A365" t="n">
+        <v>364</v>
+      </c>
+      <c r="B365" t="inlineStr"/>
+      <c r="C365" t="inlineStr"/>
+      <c r="D365" t="inlineStr"/>
+      <c r="E365" t="inlineStr"/>
+    </row>
+    <row r="366">
+      <c r="A366" t="n">
+        <v>365</v>
+      </c>
+      <c r="B366" t="inlineStr"/>
+      <c r="C366" t="inlineStr"/>
+      <c r="D366" t="inlineStr"/>
+      <c r="E366" t="inlineStr"/>
+    </row>
+    <row r="367">
+      <c r="A367" t="n">
+        <v>366</v>
+      </c>
+      <c r="B367" t="inlineStr"/>
+      <c r="C367" t="inlineStr"/>
+      <c r="D367" t="inlineStr"/>
+      <c r="E367" t="inlineStr"/>
+    </row>
+    <row r="368">
+      <c r="A368" t="n">
+        <v>367</v>
+      </c>
+      <c r="B368" t="inlineStr"/>
+      <c r="C368" t="inlineStr"/>
+      <c r="D368" t="inlineStr"/>
+      <c r="E368" t="inlineStr"/>
+    </row>
+    <row r="369">
+      <c r="A369" t="n">
+        <v>368</v>
+      </c>
+      <c r="B369" t="inlineStr"/>
+      <c r="C369" t="inlineStr"/>
+      <c r="D369" t="inlineStr"/>
+      <c r="E369" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:BH87"/>

</xml_diff>